<commit_message>
add gantt-chart and prototype-report
</commit_message>
<xml_diff>
--- a/docs/gantt-chart-risktrace.xlsx
+++ b/docs/gantt-chart-risktrace.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29DA02EA-70F7-4D42-8251-F64F77F6AEE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95231CFD-7E56-4B5C-9B3B-C22F90E02F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1114,6 +1114,21 @@
     <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1125,21 +1140,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1744,135 +1744,135 @@
       <c r="F1" s="22"/>
       <c r="H1" s="2"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="77"/>
-      <c r="W1" s="77"/>
-      <c r="X1" s="77"/>
-      <c r="Y1" s="77"/>
-      <c r="Z1" s="77"/>
-      <c r="AA1" s="77"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="82"/>
+      <c r="T1" s="82"/>
+      <c r="U1" s="82"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="82"/>
+      <c r="X1" s="82"/>
+      <c r="Y1" s="82"/>
+      <c r="Z1" s="82"/>
+      <c r="AA1" s="82"/>
     </row>
     <row r="2" spans="1:64" ht="38" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="74" t="s">
+      <c r="B2" s="79" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="74"/>
+      <c r="C2" s="79"/>
       <c r="D2" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="81">
+      <c r="E2" s="77">
         <v>46237</v>
       </c>
-      <c r="F2" s="82"/>
+      <c r="F2" s="78"/>
     </row>
     <row r="3" spans="1:64" ht="43" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="75"/>
+      <c r="C3" s="80"/>
       <c r="D3" s="61" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="81">
+      <c r="E3" s="77">
         <v>46278</v>
       </c>
-      <c r="F3" s="82"/>
+      <c r="F3" s="78"/>
     </row>
     <row r="4" spans="1:64" ht="43" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
+      <c r="B4" s="80"/>
+      <c r="C4" s="80"/>
       <c r="E4"/>
-      <c r="I4" s="78">
+      <c r="I4" s="74">
         <f>I5</f>
         <v>46237</v>
       </c>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="80"/>
-      <c r="P4" s="78">
+      <c r="J4" s="75"/>
+      <c r="K4" s="75"/>
+      <c r="L4" s="75"/>
+      <c r="M4" s="75"/>
+      <c r="N4" s="75"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="74">
         <f>P5</f>
         <v>46244</v>
       </c>
-      <c r="Q4" s="79"/>
-      <c r="R4" s="79"/>
-      <c r="S4" s="79"/>
-      <c r="T4" s="79"/>
-      <c r="U4" s="79"/>
-      <c r="V4" s="80"/>
-      <c r="W4" s="78">
+      <c r="Q4" s="75"/>
+      <c r="R4" s="75"/>
+      <c r="S4" s="75"/>
+      <c r="T4" s="75"/>
+      <c r="U4" s="75"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="74">
         <f>W5</f>
         <v>46251</v>
       </c>
-      <c r="X4" s="79"/>
-      <c r="Y4" s="79"/>
-      <c r="Z4" s="79"/>
-      <c r="AA4" s="79"/>
-      <c r="AB4" s="79"/>
-      <c r="AC4" s="80"/>
-      <c r="AD4" s="78">
+      <c r="X4" s="75"/>
+      <c r="Y4" s="75"/>
+      <c r="Z4" s="75"/>
+      <c r="AA4" s="75"/>
+      <c r="AB4" s="75"/>
+      <c r="AC4" s="76"/>
+      <c r="AD4" s="74">
         <f>AD5</f>
         <v>46258</v>
       </c>
-      <c r="AE4" s="79"/>
-      <c r="AF4" s="79"/>
-      <c r="AG4" s="79"/>
-      <c r="AH4" s="79"/>
-      <c r="AI4" s="79"/>
-      <c r="AJ4" s="80"/>
-      <c r="AK4" s="78">
+      <c r="AE4" s="75"/>
+      <c r="AF4" s="75"/>
+      <c r="AG4" s="75"/>
+      <c r="AH4" s="75"/>
+      <c r="AI4" s="75"/>
+      <c r="AJ4" s="76"/>
+      <c r="AK4" s="74">
         <f>AK5</f>
         <v>46265</v>
       </c>
-      <c r="AL4" s="79"/>
-      <c r="AM4" s="79"/>
-      <c r="AN4" s="79"/>
-      <c r="AO4" s="79"/>
-      <c r="AP4" s="79"/>
-      <c r="AQ4" s="80"/>
-      <c r="AR4" s="78">
+      <c r="AL4" s="75"/>
+      <c r="AM4" s="75"/>
+      <c r="AN4" s="75"/>
+      <c r="AO4" s="75"/>
+      <c r="AP4" s="75"/>
+      <c r="AQ4" s="76"/>
+      <c r="AR4" s="74">
         <f>AR5</f>
         <v>46272</v>
       </c>
-      <c r="AS4" s="79"/>
-      <c r="AT4" s="79"/>
-      <c r="AU4" s="79"/>
-      <c r="AV4" s="79"/>
-      <c r="AW4" s="79"/>
-      <c r="AX4" s="80"/>
-      <c r="AY4" s="78">
+      <c r="AS4" s="75"/>
+      <c r="AT4" s="75"/>
+      <c r="AU4" s="75"/>
+      <c r="AV4" s="75"/>
+      <c r="AW4" s="75"/>
+      <c r="AX4" s="76"/>
+      <c r="AY4" s="74">
         <f>AY5</f>
         <v>46279</v>
       </c>
-      <c r="AZ4" s="79"/>
-      <c r="BA4" s="79"/>
-      <c r="BB4" s="79"/>
-      <c r="BC4" s="79"/>
-      <c r="BD4" s="79"/>
-      <c r="BE4" s="80"/>
-      <c r="BF4" s="78">
+      <c r="AZ4" s="75"/>
+      <c r="BA4" s="75"/>
+      <c r="BB4" s="75"/>
+      <c r="BC4" s="75"/>
+      <c r="BD4" s="75"/>
+      <c r="BE4" s="76"/>
+      <c r="BF4" s="74">
         <f>BF5</f>
         <v>46286</v>
       </c>
-      <c r="BG4" s="79"/>
-      <c r="BH4" s="79"/>
-      <c r="BI4" s="79"/>
-      <c r="BJ4" s="79"/>
-      <c r="BK4" s="79"/>
-      <c r="BL4" s="80"/>
+      <c r="BG4" s="75"/>
+      <c r="BH4" s="75"/>
+      <c r="BI4" s="75"/>
+      <c r="BJ4" s="75"/>
+      <c r="BK4" s="75"/>
+      <c r="BL4" s="76"/>
     </row>
     <row r="5" spans="1:64" ht="23" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="6"/>
@@ -5186,7 +5186,7 @@
         <v>40</v>
       </c>
       <c r="C43" s="66" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D43" s="38">
         <v>1</v>
@@ -5270,6 +5270,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C4"/>
+    <mergeCell ref="J1:AA1"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E2:F2"/>
@@ -5278,11 +5283,6 @@
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C4"/>
-    <mergeCell ref="J1:AA1"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D43">
     <cfRule type="dataBar" priority="12">

</xml_diff>